<commit_message>
Creacion de nuevos metodos y arreglos
</commit_message>
<xml_diff>
--- a/myapp/src/main/resources/Libro3.xlsx
+++ b/myapp/src/main/resources/Libro3.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Desktop\App_TecnoMat\app_lectorArchivos\myapp\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B6DFF314-7A45-48C4-B339-E31418C1EA52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F9D1618-A3A5-40A5-886F-D6B29C152605}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{501981FC-E882-4770-BB78-4C8F6F42D128}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="71">
   <si>
     <t xml:space="preserve"> </t>
   </si>
@@ -229,6 +229,18 @@
   </si>
   <si>
     <t>Fijación s/perfilDPX³250 3P/4P</t>
+  </si>
+  <si>
+    <t>Linea cottage 43</t>
+  </si>
+  <si>
+    <t>Granja Rinya</t>
+  </si>
+  <si>
+    <t>TS260001036</t>
+  </si>
+  <si>
+    <t>LISTADO MATERIALES CE</t>
   </si>
 </sst>
 </file>
@@ -238,7 +250,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="\O\T0"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -289,6 +301,11 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <name val="Helv"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -310,7 +327,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -454,11 +471,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -477,12 +503,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -515,30 +535,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -556,12 +552,6 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -572,6 +562,45 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -588,125 +617,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>109900</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>36635</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>312854</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>14654</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="2 Imagen" descr="LOGO TECNOMAT.GIF">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{69F5A647-B2F5-4AEC-89D8-0AAA07F659B2}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="8063275" y="36635"/>
-          <a:ext cx="2488954" cy="930519"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>725366</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>109904</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>3194539</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>315058</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="3" name="CuadroTexto 2">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{95A01656-6D63-411F-B12B-9B15B2FB34E3}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="2249366" y="109904"/>
-          <a:ext cx="4183673" cy="367079"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="lt1"/>
-        </a:solidFill>
-        <a:ln w="9525" cmpd="sng">
-          <a:solidFill>
-            <a:schemeClr val="lt1">
-              <a:shade val="50000"/>
-            </a:schemeClr>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:r>
-            <a:rPr lang="es-ES" sz="2400" b="1"/>
-            <a:t>LISTADO MATERIALES CE</a:t>
-          </a:r>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -758,20 +668,10 @@
       <sheetName val="Coste Horas Cliente"/>
     </sheetNames>
     <sheetDataSet>
-      <sheetData sheetId="0">
+      <sheetData sheetId="0" refreshError="1">
         <row r="3">
           <cell r="Q3" t="str">
             <v>CE</v>
-          </cell>
-        </row>
-        <row r="11">
-          <cell r="D11" t="str">
-            <v>GRANJA RINYA</v>
-          </cell>
-        </row>
-        <row r="12">
-          <cell r="D12" t="str">
-            <v>CU DISTRIBUCION LINEA COTTAGE</v>
           </cell>
         </row>
         <row r="17">
@@ -780,45 +680,45 @@
           </cell>
         </row>
       </sheetData>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6"/>
-      <sheetData sheetId="7"/>
-      <sheetData sheetId="8"/>
-      <sheetData sheetId="9"/>
-      <sheetData sheetId="10"/>
-      <sheetData sheetId="11"/>
-      <sheetData sheetId="12"/>
-      <sheetData sheetId="13"/>
-      <sheetData sheetId="14"/>
-      <sheetData sheetId="15"/>
-      <sheetData sheetId="16"/>
-      <sheetData sheetId="17"/>
-      <sheetData sheetId="18"/>
-      <sheetData sheetId="19"/>
-      <sheetData sheetId="20"/>
-      <sheetData sheetId="21"/>
-      <sheetData sheetId="22"/>
-      <sheetData sheetId="23"/>
-      <sheetData sheetId="24"/>
-      <sheetData sheetId="25"/>
-      <sheetData sheetId="26"/>
-      <sheetData sheetId="27"/>
-      <sheetData sheetId="28"/>
-      <sheetData sheetId="29"/>
-      <sheetData sheetId="30"/>
-      <sheetData sheetId="31"/>
-      <sheetData sheetId="32"/>
-      <sheetData sheetId="33"/>
-      <sheetData sheetId="34"/>
-      <sheetData sheetId="35"/>
-      <sheetData sheetId="36"/>
-      <sheetData sheetId="37"/>
-      <sheetData sheetId="38"/>
-      <sheetData sheetId="39"/>
+      <sheetData sheetId="1" refreshError="1"/>
+      <sheetData sheetId="2" refreshError="1"/>
+      <sheetData sheetId="3" refreshError="1"/>
+      <sheetData sheetId="4" refreshError="1"/>
+      <sheetData sheetId="5" refreshError="1"/>
+      <sheetData sheetId="6" refreshError="1"/>
+      <sheetData sheetId="7" refreshError="1"/>
+      <sheetData sheetId="8" refreshError="1"/>
+      <sheetData sheetId="9" refreshError="1"/>
+      <sheetData sheetId="10" refreshError="1"/>
+      <sheetData sheetId="11" refreshError="1"/>
+      <sheetData sheetId="12" refreshError="1"/>
+      <sheetData sheetId="13" refreshError="1"/>
+      <sheetData sheetId="14" refreshError="1"/>
+      <sheetData sheetId="15" refreshError="1"/>
+      <sheetData sheetId="16" refreshError="1"/>
+      <sheetData sheetId="17" refreshError="1"/>
+      <sheetData sheetId="18" refreshError="1"/>
+      <sheetData sheetId="19" refreshError="1"/>
+      <sheetData sheetId="20" refreshError="1"/>
+      <sheetData sheetId="21" refreshError="1"/>
+      <sheetData sheetId="22" refreshError="1"/>
+      <sheetData sheetId="23" refreshError="1"/>
+      <sheetData sheetId="24" refreshError="1"/>
+      <sheetData sheetId="25" refreshError="1"/>
+      <sheetData sheetId="26" refreshError="1"/>
+      <sheetData sheetId="27" refreshError="1"/>
+      <sheetData sheetId="28" refreshError="1"/>
+      <sheetData sheetId="29" refreshError="1"/>
+      <sheetData sheetId="30" refreshError="1"/>
+      <sheetData sheetId="31" refreshError="1"/>
+      <sheetData sheetId="32" refreshError="1"/>
+      <sheetData sheetId="33" refreshError="1"/>
+      <sheetData sheetId="34" refreshError="1"/>
+      <sheetData sheetId="35" refreshError="1"/>
+      <sheetData sheetId="36" refreshError="1"/>
+      <sheetData sheetId="37" refreshError="1"/>
+      <sheetData sheetId="38" refreshError="1"/>
+      <sheetData sheetId="39" refreshError="1"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -1123,6 +1023,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F1A8B88-0AFC-458C-BD32-B938E8DB4581}">
   <dimension ref="A1:J61"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="4" max="4" width="19.5703125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
@@ -1144,91 +1047,91 @@
       </c>
       <c r="B2" s="7"/>
       <c r="C2" s="7"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="9"/>
-      <c r="F2" s="7"/>
-      <c r="G2" s="7"/>
+      <c r="D2" s="31" t="s">
+        <v>70</v>
+      </c>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
+      <c r="G2" s="31"/>
       <c r="H2" s="7"/>
       <c r="I2" s="7"/>
-      <c r="J2" s="10"/>
+      <c r="J2" s="8"/>
     </row>
     <row r="3" spans="1:10" ht="18" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
         <v>0</v>
       </c>
       <c r="B3" s="7"/>
-      <c r="C3" s="11"/>
-      <c r="D3" s="12"/>
-      <c r="E3" s="13"/>
+      <c r="C3" s="9"/>
+      <c r="D3" s="10"/>
+      <c r="E3" s="11"/>
       <c r="F3" s="7"/>
-      <c r="G3" s="7"/>
+      <c r="G3" s="30"/>
       <c r="H3" s="7"/>
       <c r="I3" s="7"/>
-      <c r="J3" s="14"/>
+      <c r="J3" s="12"/>
     </row>
     <row r="4" spans="1:10" ht="18" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
         <v>0</v>
       </c>
       <c r="B4" s="7"/>
-      <c r="C4" s="15" t="s">
-        <v>1</v>
-      </c>
-      <c r="D4" s="16">
-        <v>260001036</v>
-      </c>
-      <c r="E4" s="17"/>
+      <c r="C4" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="D4" s="14" t="s">
+        <v>69</v>
+      </c>
+      <c r="E4" s="15"/>
       <c r="F4" s="7"/>
       <c r="G4" s="7"/>
       <c r="H4" s="7"/>
-      <c r="I4" s="18"/>
-      <c r="J4" s="19"/>
-    </row>
-    <row r="5" spans="1:10" ht="54" x14ac:dyDescent="0.25">
+      <c r="I4" s="16"/>
+      <c r="J4" s="17"/>
+    </row>
+    <row r="5" spans="1:10" ht="18" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>0</v>
       </c>
       <c r="B5" s="7"/>
-      <c r="C5" s="15" t="s">
+      <c r="C5" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="20" t="str">
-        <f>'[1]OFERTA PARA EL CLIENTE'!$D$11</f>
-        <v>GRANJA RINYA</v>
-      </c>
-      <c r="E5" s="21"/>
+      <c r="D5" s="18" t="s">
+        <v>68</v>
+      </c>
+      <c r="E5" s="19"/>
       <c r="F5" s="7"/>
-      <c r="G5" s="22" t="s">
+      <c r="G5" s="34" t="s">
         <v>3</v>
       </c>
-      <c r="H5" s="22"/>
-      <c r="I5" s="23" t="s">
+      <c r="H5" s="34"/>
+      <c r="I5" s="35" t="s">
         <v>4</v>
       </c>
-      <c r="J5" s="24"/>
+      <c r="J5" s="36"/>
     </row>
     <row r="6" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>0</v>
       </c>
       <c r="B6" s="7"/>
-      <c r="C6" s="15" t="s">
+      <c r="C6" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="D6" s="25" t="str">
-        <f>CONCATENATE('[1]OFERTA PARA EL CLIENTE'!Q3," ",'[1]OFERTA PARA EL CLIENTE'!D12)</f>
-        <v>CE CU DISTRIBUCION LINEA COTTAGE</v>
-      </c>
-      <c r="E6" s="7"/>
+      <c r="D6" s="41" t="s">
+        <v>67</v>
+      </c>
+      <c r="E6" s="42"/>
       <c r="F6" s="7"/>
-      <c r="G6" s="26" t="s">
+      <c r="G6" s="37" t="s">
         <v>6</v>
       </c>
-      <c r="H6" s="26"/>
-      <c r="I6" s="27">
+      <c r="H6" s="37"/>
+      <c r="I6" s="38">
         <v>46065</v>
       </c>
-      <c r="J6" s="28"/>
+      <c r="J6" s="39"/>
     </row>
     <row r="7" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" s="6"/>
@@ -1237,1355 +1140,1356 @@
       <c r="D7" s="7"/>
       <c r="E7" s="7"/>
       <c r="F7" s="7"/>
-      <c r="G7" s="29" t="s">
+      <c r="G7" s="40" t="s">
         <v>7</v>
       </c>
-      <c r="H7" s="29"/>
-      <c r="I7" s="27">
+      <c r="H7" s="40"/>
+      <c r="I7" s="38">
         <v>46072</v>
       </c>
-      <c r="J7" s="28"/>
+      <c r="J7" s="39"/>
     </row>
     <row r="8" spans="1:10" ht="18" x14ac:dyDescent="0.25">
-      <c r="A8" s="30" t="s">
+      <c r="A8" s="20" t="s">
         <v>0</v>
       </c>
       <c r="B8" s="7"/>
-      <c r="C8" s="31"/>
-      <c r="D8" s="31"/>
-      <c r="E8" s="32"/>
-      <c r="F8" s="33"/>
-      <c r="G8" s="33"/>
-      <c r="H8" s="33"/>
-      <c r="I8" s="33"/>
-      <c r="J8" s="34"/>
+      <c r="C8" s="21"/>
+      <c r="D8" s="21"/>
+      <c r="E8" s="22"/>
+      <c r="F8" s="23"/>
+      <c r="G8" s="23"/>
+      <c r="H8" s="23"/>
+      <c r="I8" s="23"/>
+      <c r="J8" s="24"/>
     </row>
     <row r="9" spans="1:10" ht="24" x14ac:dyDescent="0.25">
-      <c r="A9" s="35" t="s">
+      <c r="A9" s="25" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="35" t="s">
+      <c r="B9" s="25" t="s">
         <v>9</v>
       </c>
-      <c r="C9" s="35" t="s">
+      <c r="C9" s="25" t="s">
         <v>10</v>
       </c>
-      <c r="D9" s="35" t="s">
+      <c r="D9" s="25" t="s">
         <v>11</v>
       </c>
-      <c r="E9" s="36" t="s">
+      <c r="E9" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="F9" s="37"/>
-      <c r="G9" s="36" t="s">
+      <c r="F9" s="33"/>
+      <c r="G9" s="32" t="s">
         <v>13</v>
       </c>
-      <c r="H9" s="37"/>
-      <c r="I9" s="38" t="s">
+      <c r="H9" s="33"/>
+      <c r="I9" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="J9" s="35" t="s">
+      <c r="J9" s="25" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A10" s="39">
+      <c r="A10" s="27">
         <v>76666</v>
       </c>
-      <c r="B10" s="39" t="s">
+      <c r="B10" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="C10" s="39" t="s">
+      <c r="C10" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="D10" s="40" t="s">
+      <c r="D10" s="28" t="s">
         <v>18</v>
       </c>
-      <c r="E10" s="41">
-        <v>1</v>
-      </c>
-      <c r="F10" s="39"/>
-      <c r="G10" s="39"/>
-      <c r="H10" s="39"/>
-      <c r="I10" s="39">
+      <c r="E10" s="29">
+        <v>1</v>
+      </c>
+      <c r="F10" s="27"/>
+      <c r="G10" s="27"/>
+      <c r="H10" s="27"/>
+      <c r="I10" s="27">
         <f>E10*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>1</v>
       </c>
-      <c r="J10" s="40"/>
+      <c r="J10" s="28"/>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A11" s="39">
+      <c r="A11" s="27">
         <v>76665</v>
       </c>
-      <c r="B11" s="39" t="s">
+      <c r="B11" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="39" t="s">
+      <c r="C11" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="D11" s="40" t="s">
+      <c r="D11" s="28" t="s">
         <v>20</v>
       </c>
-      <c r="E11" s="41">
-        <v>1</v>
-      </c>
-      <c r="F11" s="39"/>
-      <c r="G11" s="39"/>
-      <c r="H11" s="39"/>
-      <c r="I11" s="39">
+      <c r="E11" s="29">
+        <v>1</v>
+      </c>
+      <c r="F11" s="27"/>
+      <c r="G11" s="27"/>
+      <c r="H11" s="27"/>
+      <c r="I11" s="27">
         <f>E11*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>1</v>
       </c>
-      <c r="J11" s="40"/>
+      <c r="J11" s="28"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A12" s="39">
+      <c r="A12" s="27">
         <v>75884</v>
       </c>
-      <c r="B12" s="39" t="s">
+      <c r="B12" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="C12" s="39">
+      <c r="C12" s="27">
         <v>607287</v>
       </c>
-      <c r="D12" s="40" t="s">
+      <c r="D12" s="28" t="s">
         <v>21</v>
       </c>
-      <c r="E12" s="41">
-        <v>1</v>
-      </c>
-      <c r="F12" s="39"/>
-      <c r="G12" s="39"/>
-      <c r="H12" s="39"/>
-      <c r="I12" s="39">
+      <c r="E12" s="29">
+        <v>1</v>
+      </c>
+      <c r="F12" s="27"/>
+      <c r="G12" s="27"/>
+      <c r="H12" s="27"/>
+      <c r="I12" s="27">
         <f>E12*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>1</v>
       </c>
-      <c r="J12" s="40"/>
+      <c r="J12" s="28"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A13" s="39">
+      <c r="A13" s="27">
         <v>73809</v>
       </c>
-      <c r="B13" s="39" t="s">
+      <c r="B13" s="27" t="s">
         <v>22</v>
       </c>
-      <c r="C13" s="39">
+      <c r="C13" s="27">
         <v>534017</v>
       </c>
-      <c r="D13" s="40" t="s">
+      <c r="D13" s="28" t="s">
         <v>23</v>
       </c>
-      <c r="E13" s="41">
+      <c r="E13" s="29">
         <v>4</v>
       </c>
-      <c r="F13" s="39"/>
-      <c r="G13" s="39"/>
-      <c r="H13" s="39"/>
-      <c r="I13" s="39">
+      <c r="F13" s="27"/>
+      <c r="G13" s="27"/>
+      <c r="H13" s="27"/>
+      <c r="I13" s="27">
         <f>E13*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>4</v>
       </c>
-      <c r="J13" s="40"/>
+      <c r="J13" s="28"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A14" s="39">
+      <c r="A14" s="27">
         <v>65794</v>
       </c>
-      <c r="B14" s="39" t="s">
+      <c r="B14" s="27" t="s">
         <v>22</v>
       </c>
-      <c r="C14" s="39">
+      <c r="C14" s="27">
         <v>550290</v>
       </c>
-      <c r="D14" s="40" t="s">
+      <c r="D14" s="28" t="s">
         <v>24</v>
       </c>
-      <c r="E14" s="41">
-        <v>1</v>
-      </c>
-      <c r="F14" s="39"/>
-      <c r="G14" s="39"/>
-      <c r="H14" s="39"/>
-      <c r="I14" s="39">
+      <c r="E14" s="29">
+        <v>1</v>
+      </c>
+      <c r="F14" s="27"/>
+      <c r="G14" s="27"/>
+      <c r="H14" s="27"/>
+      <c r="I14" s="27">
         <f>E14*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>1</v>
       </c>
-      <c r="J14" s="40"/>
+      <c r="J14" s="28"/>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A15" s="39"/>
-      <c r="B15" s="39" t="s">
-        <v>25</v>
-      </c>
-      <c r="C15" s="39" t="s">
+      <c r="A15" s="27"/>
+      <c r="B15" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="C15" s="27" t="s">
         <v>26</v>
       </c>
-      <c r="D15" s="40" t="s">
+      <c r="D15" s="28" t="s">
         <v>27</v>
       </c>
-      <c r="E15" s="41">
-        <v>1</v>
-      </c>
-      <c r="F15" s="39"/>
-      <c r="G15" s="39"/>
-      <c r="H15" s="39"/>
-      <c r="I15" s="39">
+      <c r="E15" s="29">
+        <v>1</v>
+      </c>
+      <c r="F15" s="27"/>
+      <c r="G15" s="27"/>
+      <c r="H15" s="27"/>
+      <c r="I15" s="27">
         <f>E15*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>1</v>
       </c>
-      <c r="J15" s="40"/>
+      <c r="J15" s="28"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A16" s="39">
+      <c r="A16" s="27">
         <v>79562</v>
       </c>
-      <c r="B16" s="39" t="s">
-        <v>25</v>
-      </c>
-      <c r="C16" s="39">
+      <c r="B16" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="C16" s="27">
         <v>5818</v>
       </c>
-      <c r="D16" s="40" t="s">
+      <c r="D16" s="28" t="s">
         <v>28</v>
       </c>
-      <c r="E16" s="41">
+      <c r="E16" s="29">
         <v>4</v>
       </c>
-      <c r="F16" s="39"/>
-      <c r="G16" s="39"/>
-      <c r="H16" s="39"/>
-      <c r="I16" s="39">
+      <c r="F16" s="27"/>
+      <c r="G16" s="27"/>
+      <c r="H16" s="27"/>
+      <c r="I16" s="27">
         <f>E16*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>4</v>
       </c>
-      <c r="J16" s="40"/>
+      <c r="J16" s="28"/>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A17" s="39">
+      <c r="A17" s="27">
         <v>79563</v>
       </c>
-      <c r="B17" s="39" t="s">
-        <v>25</v>
-      </c>
-      <c r="C17" s="39">
+      <c r="B17" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="C17" s="27">
         <v>13302</v>
       </c>
-      <c r="D17" s="40" t="s">
+      <c r="D17" s="28" t="s">
         <v>29</v>
       </c>
-      <c r="E17" s="41">
+      <c r="E17" s="29">
         <v>4</v>
       </c>
-      <c r="F17" s="39"/>
-      <c r="G17" s="39"/>
-      <c r="H17" s="39"/>
-      <c r="I17" s="39">
+      <c r="F17" s="27"/>
+      <c r="G17" s="27"/>
+      <c r="H17" s="27"/>
+      <c r="I17" s="27">
         <f>E17*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>4</v>
       </c>
-      <c r="J17" s="40"/>
+      <c r="J17" s="28"/>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A18" s="39">
+      <c r="A18" s="27">
         <v>79564</v>
       </c>
-      <c r="B18" s="39" t="s">
-        <v>25</v>
-      </c>
-      <c r="C18" s="39">
+      <c r="B18" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="C18" s="27">
         <v>20051</v>
       </c>
-      <c r="D18" s="40" t="s">
+      <c r="D18" s="28" t="s">
         <v>30</v>
       </c>
-      <c r="E18" s="41">
+      <c r="E18" s="29">
         <v>3</v>
       </c>
-      <c r="F18" s="39"/>
-      <c r="G18" s="39"/>
-      <c r="H18" s="39"/>
-      <c r="I18" s="39">
+      <c r="F18" s="27"/>
+      <c r="G18" s="27"/>
+      <c r="H18" s="27"/>
+      <c r="I18" s="27">
         <f>E18*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>3</v>
       </c>
-      <c r="J18" s="40"/>
+      <c r="J18" s="28"/>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A19" s="39">
+      <c r="A19" s="27">
         <v>71109</v>
       </c>
-      <c r="B19" s="39" t="s">
-        <v>25</v>
-      </c>
-      <c r="C19" s="39">
+      <c r="B19" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="C19" s="27">
         <v>20119</v>
       </c>
-      <c r="D19" s="40" t="s">
+      <c r="D19" s="28" t="s">
         <v>31</v>
       </c>
-      <c r="E19" s="41">
-        <v>1</v>
-      </c>
-      <c r="F19" s="39"/>
-      <c r="G19" s="39"/>
-      <c r="H19" s="39"/>
-      <c r="I19" s="39">
+      <c r="E19" s="29">
+        <v>1</v>
+      </c>
+      <c r="F19" s="27"/>
+      <c r="G19" s="27"/>
+      <c r="H19" s="27"/>
+      <c r="I19" s="27">
         <f>E19*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>1</v>
       </c>
-      <c r="J19" s="40"/>
+      <c r="J19" s="28"/>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A20" s="39">
+      <c r="A20" s="27">
         <v>80696</v>
       </c>
-      <c r="B20" s="39" t="s">
-        <v>25</v>
-      </c>
-      <c r="C20" s="39">
+      <c r="B20" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="C20" s="27">
         <v>20139</v>
       </c>
-      <c r="D20" s="40" t="s">
+      <c r="D20" s="28" t="s">
         <v>32</v>
       </c>
-      <c r="E20" s="41">
-        <v>1</v>
-      </c>
-      <c r="F20" s="39"/>
-      <c r="G20" s="39"/>
-      <c r="H20" s="39"/>
-      <c r="I20" s="39">
+      <c r="E20" s="29">
+        <v>1</v>
+      </c>
+      <c r="F20" s="27"/>
+      <c r="G20" s="27"/>
+      <c r="H20" s="27"/>
+      <c r="I20" s="27">
         <f>E20*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>1</v>
       </c>
-      <c r="J20" s="40"/>
+      <c r="J20" s="28"/>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A21" s="39">
+      <c r="A21" s="27">
         <v>80697</v>
       </c>
-      <c r="B21" s="39" t="s">
-        <v>25</v>
-      </c>
-      <c r="C21" s="39">
+      <c r="B21" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="C21" s="27">
         <v>20149</v>
       </c>
-      <c r="D21" s="40" t="s">
+      <c r="D21" s="28" t="s">
         <v>33</v>
       </c>
-      <c r="E21" s="41">
-        <v>1</v>
-      </c>
-      <c r="F21" s="39"/>
-      <c r="G21" s="39"/>
-      <c r="H21" s="39"/>
-      <c r="I21" s="39">
+      <c r="E21" s="29">
+        <v>1</v>
+      </c>
+      <c r="F21" s="27"/>
+      <c r="G21" s="27"/>
+      <c r="H21" s="27"/>
+      <c r="I21" s="27">
         <f>E21*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>1</v>
       </c>
-      <c r="J21" s="40"/>
+      <c r="J21" s="28"/>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A22" s="39">
+      <c r="A22" s="27">
         <v>80698</v>
       </c>
-      <c r="B22" s="39" t="s">
-        <v>25</v>
-      </c>
-      <c r="C22" s="39">
+      <c r="B22" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="C22" s="27">
         <v>20169</v>
       </c>
-      <c r="D22" s="40" t="s">
+      <c r="D22" s="28" t="s">
         <v>34</v>
       </c>
-      <c r="E22" s="41">
-        <v>1</v>
-      </c>
-      <c r="F22" s="39"/>
-      <c r="G22" s="39"/>
-      <c r="H22" s="39"/>
-      <c r="I22" s="39">
+      <c r="E22" s="29">
+        <v>1</v>
+      </c>
+      <c r="F22" s="27"/>
+      <c r="G22" s="27"/>
+      <c r="H22" s="27"/>
+      <c r="I22" s="27">
         <f>E22*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>1</v>
       </c>
-      <c r="J22" s="40"/>
+      <c r="J22" s="28"/>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A23" s="39">
+      <c r="A23" s="27">
         <v>79672</v>
       </c>
-      <c r="B23" s="39" t="s">
-        <v>25</v>
-      </c>
-      <c r="C23" s="39">
+      <c r="B23" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="C23" s="27">
         <v>20201</v>
       </c>
-      <c r="D23" s="40" t="s">
+      <c r="D23" s="28" t="s">
         <v>35</v>
       </c>
-      <c r="E23" s="41">
+      <c r="E23" s="29">
         <v>2</v>
       </c>
-      <c r="F23" s="39"/>
-      <c r="G23" s="39"/>
-      <c r="H23" s="39"/>
-      <c r="I23" s="39">
+      <c r="F23" s="27"/>
+      <c r="G23" s="27"/>
+      <c r="H23" s="27"/>
+      <c r="I23" s="27">
         <f>E23*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>2</v>
       </c>
-      <c r="J23" s="40"/>
+      <c r="J23" s="28"/>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A24" s="39">
+      <c r="A24" s="27">
         <v>80699</v>
       </c>
-      <c r="B24" s="39" t="s">
-        <v>25</v>
-      </c>
-      <c r="C24" s="39">
+      <c r="B24" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="C24" s="27">
         <v>20204</v>
       </c>
-      <c r="D24" s="40" t="s">
+      <c r="D24" s="28" t="s">
         <v>36</v>
       </c>
-      <c r="E24" s="41">
-        <v>1</v>
-      </c>
-      <c r="F24" s="39"/>
-      <c r="G24" s="39"/>
-      <c r="H24" s="39"/>
-      <c r="I24" s="39">
+      <c r="E24" s="29">
+        <v>1</v>
+      </c>
+      <c r="F24" s="27"/>
+      <c r="G24" s="27"/>
+      <c r="H24" s="27"/>
+      <c r="I24" s="27">
         <f>E24*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>1</v>
       </c>
-      <c r="J24" s="40"/>
+      <c r="J24" s="28"/>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A25" s="39">
+      <c r="A25" s="27">
         <v>80700</v>
       </c>
-      <c r="B25" s="39" t="s">
-        <v>25</v>
-      </c>
-      <c r="C25" s="39">
+      <c r="B25" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="C25" s="27">
         <v>20207</v>
       </c>
-      <c r="D25" s="40" t="s">
+      <c r="D25" s="28" t="s">
         <v>37</v>
       </c>
-      <c r="E25" s="41">
-        <v>1</v>
-      </c>
-      <c r="F25" s="39"/>
-      <c r="G25" s="39"/>
-      <c r="H25" s="39"/>
-      <c r="I25" s="39">
+      <c r="E25" s="29">
+        <v>1</v>
+      </c>
+      <c r="F25" s="27"/>
+      <c r="G25" s="27"/>
+      <c r="H25" s="27"/>
+      <c r="I25" s="27">
         <f>E25*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>1</v>
       </c>
-      <c r="J25" s="40"/>
+      <c r="J25" s="28"/>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A26" s="39">
+      <c r="A26" s="27">
         <v>80701</v>
       </c>
-      <c r="B26" s="39" t="s">
-        <v>25</v>
-      </c>
-      <c r="C26" s="39">
+      <c r="B26" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="C26" s="27">
         <v>20211</v>
       </c>
-      <c r="D26" s="40" t="s">
+      <c r="D26" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="E26" s="41">
+      <c r="E26" s="29">
         <v>2</v>
       </c>
-      <c r="F26" s="39"/>
-      <c r="G26" s="39"/>
-      <c r="H26" s="39"/>
-      <c r="I26" s="39">
+      <c r="F26" s="27"/>
+      <c r="G26" s="27"/>
+      <c r="H26" s="27"/>
+      <c r="I26" s="27">
         <f>E26*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>2</v>
       </c>
-      <c r="J26" s="40"/>
+      <c r="J26" s="28"/>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A27" s="39">
+      <c r="A27" s="27">
         <v>80702</v>
       </c>
-      <c r="B27" s="39" t="s">
-        <v>25</v>
-      </c>
-      <c r="C27" s="39">
+      <c r="B27" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="C27" s="27">
         <v>20279</v>
       </c>
-      <c r="D27" s="40" t="s">
+      <c r="D27" s="28" t="s">
         <v>39</v>
       </c>
-      <c r="E27" s="41">
-        <v>1</v>
-      </c>
-      <c r="F27" s="39"/>
-      <c r="G27" s="39"/>
-      <c r="H27" s="39"/>
-      <c r="I27" s="39">
+      <c r="E27" s="29">
+        <v>1</v>
+      </c>
+      <c r="F27" s="27"/>
+      <c r="G27" s="27"/>
+      <c r="H27" s="27"/>
+      <c r="I27" s="27">
         <f>E27*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>1</v>
       </c>
-      <c r="J27" s="40"/>
+      <c r="J27" s="28"/>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A28" s="39">
+      <c r="A28" s="27">
         <v>79565</v>
       </c>
-      <c r="B28" s="39" t="s">
-        <v>25</v>
-      </c>
-      <c r="C28" s="39">
+      <c r="B28" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="C28" s="27">
         <v>20291</v>
       </c>
-      <c r="D28" s="40" t="s">
+      <c r="D28" s="28" t="s">
         <v>40</v>
       </c>
-      <c r="E28" s="41">
+      <c r="E28" s="29">
         <v>2</v>
       </c>
-      <c r="F28" s="39"/>
-      <c r="G28" s="39"/>
-      <c r="H28" s="39"/>
-      <c r="I28" s="39">
+      <c r="F28" s="27"/>
+      <c r="G28" s="27"/>
+      <c r="H28" s="27"/>
+      <c r="I28" s="27">
         <f>E28*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>2</v>
       </c>
-      <c r="J28" s="40"/>
+      <c r="J28" s="28"/>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A29" s="39">
+      <c r="A29" s="27">
         <v>79671</v>
       </c>
-      <c r="B29" s="39" t="s">
-        <v>25</v>
-      </c>
-      <c r="C29" s="39">
+      <c r="B29" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="C29" s="27">
         <v>20300</v>
       </c>
-      <c r="D29" s="40" t="s">
+      <c r="D29" s="28" t="s">
         <v>41</v>
       </c>
-      <c r="E29" s="41">
+      <c r="E29" s="29">
         <v>2</v>
       </c>
-      <c r="F29" s="39"/>
-      <c r="G29" s="39"/>
-      <c r="H29" s="39"/>
-      <c r="I29" s="39">
+      <c r="F29" s="27"/>
+      <c r="G29" s="27"/>
+      <c r="H29" s="27"/>
+      <c r="I29" s="27">
         <f>E29*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>2</v>
       </c>
-      <c r="J29" s="40"/>
+      <c r="J29" s="28"/>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A30" s="39">
+      <c r="A30" s="27">
         <v>80703</v>
       </c>
-      <c r="B30" s="39" t="s">
-        <v>25</v>
-      </c>
-      <c r="C30" s="39">
+      <c r="B30" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="C30" s="27">
         <v>20307</v>
       </c>
-      <c r="D30" s="40" t="s">
+      <c r="D30" s="28" t="s">
         <v>42</v>
       </c>
-      <c r="E30" s="41">
-        <v>1</v>
-      </c>
-      <c r="F30" s="39"/>
-      <c r="G30" s="39"/>
-      <c r="H30" s="39"/>
-      <c r="I30" s="39">
+      <c r="E30" s="29">
+        <v>1</v>
+      </c>
+      <c r="F30" s="27"/>
+      <c r="G30" s="27"/>
+      <c r="H30" s="27"/>
+      <c r="I30" s="27">
         <f>E30*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>1</v>
       </c>
-      <c r="J30" s="40"/>
+      <c r="J30" s="28"/>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A31" s="39">
+      <c r="A31" s="27">
         <v>80704</v>
       </c>
-      <c r="B31" s="39" t="s">
-        <v>25</v>
-      </c>
-      <c r="C31" s="39">
+      <c r="B31" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="C31" s="27">
         <v>20310</v>
       </c>
-      <c r="D31" s="40" t="s">
+      <c r="D31" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="E31" s="41">
+      <c r="E31" s="29">
         <v>2</v>
       </c>
-      <c r="F31" s="39"/>
-      <c r="G31" s="39"/>
-      <c r="H31" s="39"/>
-      <c r="I31" s="39">
+      <c r="F31" s="27"/>
+      <c r="G31" s="27"/>
+      <c r="H31" s="27"/>
+      <c r="I31" s="27">
         <f>E31*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>2</v>
       </c>
-      <c r="J31" s="40"/>
+      <c r="J31" s="28"/>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A32" s="39">
+      <c r="A32" s="27">
         <v>79845</v>
       </c>
-      <c r="B32" s="39" t="s">
-        <v>25</v>
-      </c>
-      <c r="C32" s="39">
+      <c r="B32" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="C32" s="27">
         <v>20342</v>
       </c>
-      <c r="D32" s="40" t="s">
+      <c r="D32" s="28" t="s">
         <v>44</v>
       </c>
-      <c r="E32" s="41">
-        <v>1</v>
-      </c>
-      <c r="F32" s="39"/>
-      <c r="G32" s="39"/>
-      <c r="H32" s="39"/>
-      <c r="I32" s="39">
+      <c r="E32" s="29">
+        <v>1</v>
+      </c>
+      <c r="F32" s="27"/>
+      <c r="G32" s="27"/>
+      <c r="H32" s="27"/>
+      <c r="I32" s="27">
         <f>E32*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>1</v>
       </c>
-      <c r="J32" s="40"/>
+      <c r="J32" s="28"/>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A33" s="39">
+      <c r="A33" s="27">
         <v>80705</v>
       </c>
-      <c r="B33" s="39" t="s">
-        <v>25</v>
-      </c>
-      <c r="C33" s="39">
+      <c r="B33" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="C33" s="27">
         <v>20343</v>
       </c>
-      <c r="D33" s="40" t="s">
+      <c r="D33" s="28" t="s">
         <v>45</v>
       </c>
-      <c r="E33" s="41">
+      <c r="E33" s="29">
         <v>2</v>
       </c>
-      <c r="F33" s="39"/>
-      <c r="G33" s="39"/>
-      <c r="H33" s="39"/>
-      <c r="I33" s="39">
+      <c r="F33" s="27"/>
+      <c r="G33" s="27"/>
+      <c r="H33" s="27"/>
+      <c r="I33" s="27">
         <f>E33*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>2</v>
       </c>
-      <c r="J33" s="40"/>
+      <c r="J33" s="28"/>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A34" s="39">
+      <c r="A34" s="27">
         <v>79582</v>
       </c>
-      <c r="B34" s="39" t="s">
-        <v>25</v>
-      </c>
-      <c r="C34" s="39">
+      <c r="B34" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="C34" s="27">
         <v>26088</v>
       </c>
-      <c r="D34" s="40" t="s">
+      <c r="D34" s="28" t="s">
         <v>46</v>
       </c>
-      <c r="E34" s="41">
+      <c r="E34" s="29">
         <v>4</v>
       </c>
-      <c r="F34" s="39"/>
-      <c r="G34" s="39"/>
-      <c r="H34" s="39"/>
-      <c r="I34" s="39">
+      <c r="F34" s="27"/>
+      <c r="G34" s="27"/>
+      <c r="H34" s="27"/>
+      <c r="I34" s="27">
         <f>E34*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>4</v>
       </c>
-      <c r="J34" s="40"/>
+      <c r="J34" s="28"/>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A35" s="39">
+      <c r="A35" s="27">
         <v>79670</v>
       </c>
-      <c r="B35" s="39" t="s">
-        <v>25</v>
-      </c>
-      <c r="C35" s="39">
+      <c r="B35" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="C35" s="27">
         <v>26092</v>
       </c>
-      <c r="D35" s="40" t="s">
+      <c r="D35" s="28" t="s">
         <v>47</v>
       </c>
-      <c r="E35" s="41">
+      <c r="E35" s="29">
         <v>3</v>
       </c>
-      <c r="F35" s="39"/>
-      <c r="G35" s="39"/>
-      <c r="H35" s="39"/>
-      <c r="I35" s="39">
+      <c r="F35" s="27"/>
+      <c r="G35" s="27"/>
+      <c r="H35" s="27"/>
+      <c r="I35" s="27">
         <f>E35*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>3</v>
       </c>
-      <c r="J35" s="40"/>
+      <c r="J35" s="28"/>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A36" s="39">
+      <c r="A36" s="27">
         <v>79583</v>
       </c>
-      <c r="B36" s="39" t="s">
-        <v>25</v>
-      </c>
-      <c r="C36" s="39">
+      <c r="B36" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="C36" s="27">
         <v>26093</v>
       </c>
-      <c r="D36" s="40" t="s">
+      <c r="D36" s="28" t="s">
         <v>48</v>
       </c>
-      <c r="E36" s="41">
-        <v>1</v>
-      </c>
-      <c r="F36" s="39"/>
-      <c r="G36" s="39"/>
-      <c r="H36" s="39"/>
-      <c r="I36" s="39">
+      <c r="E36" s="29">
+        <v>1</v>
+      </c>
+      <c r="F36" s="27"/>
+      <c r="G36" s="27"/>
+      <c r="H36" s="27"/>
+      <c r="I36" s="27">
         <f>E36*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>1</v>
       </c>
-      <c r="J36" s="40"/>
+      <c r="J36" s="28"/>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A37" s="39">
+      <c r="A37" s="27">
         <v>79584</v>
       </c>
-      <c r="B37" s="39" t="s">
-        <v>25</v>
-      </c>
-      <c r="C37" s="39">
+      <c r="B37" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="C37" s="27">
         <v>26249</v>
       </c>
-      <c r="D37" s="40" t="s">
+      <c r="D37" s="28" t="s">
         <v>49</v>
       </c>
-      <c r="E37" s="41">
-        <v>1</v>
-      </c>
-      <c r="F37" s="39"/>
-      <c r="G37" s="39"/>
-      <c r="H37" s="39"/>
-      <c r="I37" s="39">
+      <c r="E37" s="29">
+        <v>1</v>
+      </c>
+      <c r="F37" s="27"/>
+      <c r="G37" s="27"/>
+      <c r="H37" s="27"/>
+      <c r="I37" s="27">
         <f>E37*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>1</v>
       </c>
-      <c r="J37" s="40"/>
+      <c r="J37" s="28"/>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A38" s="39">
+      <c r="A38" s="27">
         <v>79585</v>
       </c>
-      <c r="B38" s="39" t="s">
-        <v>25</v>
-      </c>
-      <c r="C38" s="39">
+      <c r="B38" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="C38" s="27">
         <v>26662</v>
       </c>
-      <c r="D38" s="40" t="s">
+      <c r="D38" s="28" t="s">
         <v>50</v>
       </c>
-      <c r="E38" s="41">
-        <v>1</v>
-      </c>
-      <c r="F38" s="39"/>
-      <c r="G38" s="39"/>
-      <c r="H38" s="39"/>
-      <c r="I38" s="39">
+      <c r="E38" s="29">
+        <v>1</v>
+      </c>
+      <c r="F38" s="27"/>
+      <c r="G38" s="27"/>
+      <c r="H38" s="27"/>
+      <c r="I38" s="27">
         <f>E38*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>1</v>
       </c>
-      <c r="J38" s="40"/>
+      <c r="J38" s="28"/>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A39" s="39">
+      <c r="A39" s="27">
         <v>71525</v>
       </c>
-      <c r="B39" s="39" t="s">
-        <v>25</v>
-      </c>
-      <c r="C39" s="39">
+      <c r="B39" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="C39" s="27">
         <v>37310</v>
       </c>
-      <c r="D39" s="40" t="s">
+      <c r="D39" s="28" t="s">
         <v>51</v>
       </c>
-      <c r="E39" s="41">
+      <c r="E39" s="29">
         <v>4</v>
       </c>
-      <c r="F39" s="39"/>
-      <c r="G39" s="39"/>
-      <c r="H39" s="39"/>
-      <c r="I39" s="39">
+      <c r="F39" s="27"/>
+      <c r="G39" s="27"/>
+      <c r="H39" s="27"/>
+      <c r="I39" s="27">
         <f>E39*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>4</v>
       </c>
-      <c r="J39" s="40"/>
+      <c r="J39" s="28"/>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A40" s="39">
+      <c r="A40" s="27">
         <v>79587</v>
       </c>
-      <c r="B40" s="39" t="s">
-        <v>25</v>
-      </c>
-      <c r="C40" s="39">
+      <c r="B40" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="C40" s="27">
         <v>37385</v>
       </c>
-      <c r="D40" s="40" t="s">
+      <c r="D40" s="28" t="s">
         <v>52</v>
       </c>
-      <c r="E40" s="41">
+      <c r="E40" s="29">
         <v>2</v>
       </c>
-      <c r="F40" s="39"/>
-      <c r="G40" s="39"/>
-      <c r="H40" s="39"/>
-      <c r="I40" s="39">
+      <c r="F40" s="27"/>
+      <c r="G40" s="27"/>
+      <c r="H40" s="27"/>
+      <c r="I40" s="27">
         <f>E40*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>2</v>
       </c>
-      <c r="J40" s="40"/>
+      <c r="J40" s="28"/>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A41" s="39">
+      <c r="A41" s="27">
         <v>79588</v>
       </c>
-      <c r="B41" s="39" t="s">
-        <v>25</v>
-      </c>
-      <c r="C41" s="39">
+      <c r="B41" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="C41" s="27">
         <v>37419</v>
       </c>
-      <c r="D41" s="40" t="s">
+      <c r="D41" s="28" t="s">
         <v>53</v>
       </c>
-      <c r="E41" s="41">
+      <c r="E41" s="29">
         <v>4</v>
       </c>
-      <c r="F41" s="39"/>
-      <c r="G41" s="39"/>
-      <c r="H41" s="39"/>
-      <c r="I41" s="39">
+      <c r="F41" s="27"/>
+      <c r="G41" s="27"/>
+      <c r="H41" s="27"/>
+      <c r="I41" s="27">
         <f>E41*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>4</v>
       </c>
-      <c r="J41" s="40"/>
+      <c r="J41" s="28"/>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A42" s="39">
+      <c r="A42" s="27">
         <v>79589</v>
       </c>
-      <c r="B42" s="39" t="s">
-        <v>25</v>
-      </c>
-      <c r="C42" s="39">
+      <c r="B42" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="C42" s="27">
         <v>37438</v>
       </c>
-      <c r="D42" s="40" t="s">
+      <c r="D42" s="28" t="s">
         <v>54</v>
       </c>
-      <c r="E42" s="41">
-        <v>1</v>
-      </c>
-      <c r="F42" s="39"/>
-      <c r="G42" s="39"/>
-      <c r="H42" s="39"/>
-      <c r="I42" s="39">
+      <c r="E42" s="29">
+        <v>1</v>
+      </c>
+      <c r="F42" s="27"/>
+      <c r="G42" s="27"/>
+      <c r="H42" s="27"/>
+      <c r="I42" s="27">
         <f>E42*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>1</v>
       </c>
-      <c r="J42" s="40"/>
+      <c r="J42" s="28"/>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A43" s="39">
+      <c r="A43" s="27">
         <v>79590</v>
       </c>
-      <c r="B43" s="39" t="s">
-        <v>25</v>
-      </c>
-      <c r="C43" s="39">
+      <c r="B43" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="C43" s="27">
         <v>405226</v>
       </c>
-      <c r="D43" s="40" t="s">
+      <c r="D43" s="28" t="s">
         <v>55</v>
       </c>
-      <c r="E43" s="41">
+      <c r="E43" s="29">
         <v>2</v>
       </c>
-      <c r="F43" s="39"/>
-      <c r="G43" s="39"/>
-      <c r="H43" s="39"/>
-      <c r="I43" s="39">
+      <c r="F43" s="27"/>
+      <c r="G43" s="27"/>
+      <c r="H43" s="27"/>
+      <c r="I43" s="27">
         <f>E43*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>2</v>
       </c>
-      <c r="J43" s="40"/>
+      <c r="J43" s="28"/>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A44" s="39">
+      <c r="A44" s="27">
         <v>70806</v>
       </c>
-      <c r="B44" s="39" t="s">
-        <v>25</v>
-      </c>
-      <c r="C44" s="39">
+      <c r="B44" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="C44" s="27">
         <v>407752</v>
       </c>
-      <c r="D44" s="40" t="s">
+      <c r="D44" s="28" t="s">
         <v>56</v>
       </c>
-      <c r="E44" s="41">
-        <v>1</v>
-      </c>
-      <c r="F44" s="39"/>
-      <c r="G44" s="39"/>
-      <c r="H44" s="39"/>
-      <c r="I44" s="39">
+      <c r="E44" s="29">
+        <v>1</v>
+      </c>
+      <c r="F44" s="27"/>
+      <c r="G44" s="27"/>
+      <c r="H44" s="27"/>
+      <c r="I44" s="27">
         <f>E44*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>1</v>
       </c>
-      <c r="J44" s="40"/>
+      <c r="J44" s="28"/>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A45" s="39">
+      <c r="A45" s="27">
         <v>79597</v>
       </c>
-      <c r="B45" s="39" t="s">
-        <v>25</v>
-      </c>
-      <c r="C45" s="39">
+      <c r="B45" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="C45" s="27">
         <v>411504</v>
       </c>
-      <c r="D45" s="40" t="s">
+      <c r="D45" s="28" t="s">
         <v>57</v>
       </c>
-      <c r="E45" s="41">
-        <v>1</v>
-      </c>
-      <c r="F45" s="39"/>
-      <c r="G45" s="39"/>
-      <c r="H45" s="39"/>
-      <c r="I45" s="39">
+      <c r="E45" s="29">
+        <v>1</v>
+      </c>
+      <c r="F45" s="27"/>
+      <c r="G45" s="27"/>
+      <c r="H45" s="27"/>
+      <c r="I45" s="27">
         <f>E45*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>1</v>
       </c>
-      <c r="J45" s="40"/>
+      <c r="J45" s="28"/>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A46" s="39">
+      <c r="A46" s="27">
         <v>80707</v>
       </c>
-      <c r="B46" s="39" t="s">
-        <v>25</v>
-      </c>
-      <c r="C46" s="39">
+      <c r="B46" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="C46" s="27">
         <v>420012</v>
       </c>
-      <c r="D46" s="40" t="s">
+      <c r="D46" s="28" t="s">
         <v>58</v>
       </c>
-      <c r="E46" s="41">
-        <v>1</v>
-      </c>
-      <c r="F46" s="39"/>
-      <c r="G46" s="39"/>
-      <c r="H46" s="39"/>
-      <c r="I46" s="39">
+      <c r="E46" s="29">
+        <v>1</v>
+      </c>
+      <c r="F46" s="27"/>
+      <c r="G46" s="27"/>
+      <c r="H46" s="27"/>
+      <c r="I46" s="27">
         <f>E46*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>1</v>
       </c>
-      <c r="J46" s="40"/>
+      <c r="J46" s="28"/>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A47" s="39">
+      <c r="A47" s="27">
         <v>80708</v>
       </c>
-      <c r="B47" s="39" t="s">
-        <v>25</v>
-      </c>
-      <c r="C47" s="39">
+      <c r="B47" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="C47" s="27">
         <v>420013</v>
       </c>
-      <c r="D47" s="40" t="s">
+      <c r="D47" s="28" t="s">
         <v>59</v>
       </c>
-      <c r="E47" s="41">
+      <c r="E47" s="29">
         <v>2</v>
       </c>
-      <c r="F47" s="39"/>
-      <c r="G47" s="39"/>
-      <c r="H47" s="39"/>
-      <c r="I47" s="39">
+      <c r="F47" s="27"/>
+      <c r="G47" s="27"/>
+      <c r="H47" s="27"/>
+      <c r="I47" s="27">
         <f>E47*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>2</v>
       </c>
-      <c r="J47" s="40"/>
+      <c r="J47" s="28"/>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A48" s="39">
+      <c r="A48" s="27">
         <v>67464</v>
       </c>
-      <c r="B48" s="39" t="s">
-        <v>25</v>
-      </c>
-      <c r="C48" s="39">
+      <c r="B48" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="C48" s="27">
         <v>420016</v>
       </c>
-      <c r="D48" s="40" t="s">
+      <c r="D48" s="28" t="s">
         <v>60</v>
       </c>
-      <c r="E48" s="41">
-        <v>1</v>
-      </c>
-      <c r="F48" s="39"/>
-      <c r="G48" s="39"/>
-      <c r="H48" s="39"/>
-      <c r="I48" s="39">
+      <c r="E48" s="29">
+        <v>1</v>
+      </c>
+      <c r="F48" s="27"/>
+      <c r="G48" s="27"/>
+      <c r="H48" s="27"/>
+      <c r="I48" s="27">
         <f>E48*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>1</v>
       </c>
-      <c r="J48" s="40"/>
+      <c r="J48" s="28"/>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A49" s="39">
+      <c r="A49" s="27">
         <v>79603</v>
       </c>
-      <c r="B49" s="39" t="s">
-        <v>25</v>
-      </c>
-      <c r="C49" s="39">
+      <c r="B49" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="C49" s="27">
         <v>421016</v>
       </c>
-      <c r="D49" s="40" t="s">
+      <c r="D49" s="28" t="s">
         <v>61</v>
       </c>
-      <c r="E49" s="41">
+      <c r="E49" s="29">
         <v>4</v>
       </c>
-      <c r="F49" s="39"/>
-      <c r="G49" s="39"/>
-      <c r="H49" s="39"/>
-      <c r="I49" s="39">
+      <c r="F49" s="27"/>
+      <c r="G49" s="27"/>
+      <c r="H49" s="27"/>
+      <c r="I49" s="27">
         <f>E49*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>4</v>
       </c>
-      <c r="J49" s="40"/>
+      <c r="J49" s="28"/>
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A50" s="39">
+      <c r="A50" s="27">
         <v>79668</v>
       </c>
-      <c r="B50" s="39" t="s">
-        <v>25</v>
-      </c>
-      <c r="C50" s="39">
+      <c r="B50" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="C50" s="27">
         <v>421071</v>
       </c>
-      <c r="D50" s="40" t="s">
+      <c r="D50" s="28" t="s">
         <v>62</v>
       </c>
-      <c r="E50" s="41">
+      <c r="E50" s="29">
         <v>4</v>
       </c>
-      <c r="F50" s="39"/>
-      <c r="G50" s="39"/>
-      <c r="H50" s="39"/>
-      <c r="I50" s="39">
+      <c r="F50" s="27"/>
+      <c r="G50" s="27"/>
+      <c r="H50" s="27"/>
+      <c r="I50" s="27">
         <f>E50*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>4</v>
       </c>
-      <c r="J50" s="40"/>
+      <c r="J50" s="28"/>
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A51" s="39">
+      <c r="A51" s="27">
         <v>79597</v>
       </c>
-      <c r="B51" s="39" t="s">
-        <v>25</v>
-      </c>
-      <c r="C51" s="39">
+      <c r="B51" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="C51" s="27">
         <v>411504</v>
       </c>
-      <c r="D51" s="40" t="s">
+      <c r="D51" s="28" t="s">
         <v>57</v>
       </c>
-      <c r="E51" s="41">
-        <v>1</v>
-      </c>
-      <c r="F51" s="39"/>
-      <c r="G51" s="39"/>
-      <c r="H51" s="39"/>
-      <c r="I51" s="39">
+      <c r="E51" s="29">
+        <v>1</v>
+      </c>
+      <c r="F51" s="27"/>
+      <c r="G51" s="27"/>
+      <c r="H51" s="27"/>
+      <c r="I51" s="27">
         <f>E51*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>1</v>
       </c>
-      <c r="J51" s="40"/>
+      <c r="J51" s="28"/>
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A52" s="39">
+      <c r="A52" s="27">
         <v>79592</v>
       </c>
-      <c r="B52" s="39" t="s">
-        <v>25</v>
-      </c>
-      <c r="C52" s="39">
+      <c r="B52" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="C52" s="27">
         <v>407800</v>
       </c>
-      <c r="D52" s="40" t="s">
+      <c r="D52" s="28" t="s">
         <v>63</v>
       </c>
-      <c r="E52" s="41">
-        <v>1</v>
-      </c>
-      <c r="F52" s="39"/>
-      <c r="G52" s="39"/>
-      <c r="H52" s="39"/>
-      <c r="I52" s="39">
+      <c r="E52" s="29">
+        <v>1</v>
+      </c>
+      <c r="F52" s="27"/>
+      <c r="G52" s="27"/>
+      <c r="H52" s="27"/>
+      <c r="I52" s="27">
         <f>E52*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>1</v>
       </c>
-      <c r="J52" s="40"/>
+      <c r="J52" s="28"/>
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A53" s="39"/>
-      <c r="B53" s="39" t="s">
-        <v>25</v>
-      </c>
-      <c r="C53" s="39" t="s">
+      <c r="A53" s="27"/>
+      <c r="B53" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="C53" s="27" t="s">
         <v>26</v>
       </c>
-      <c r="D53" s="40" t="s">
+      <c r="D53" s="28" t="s">
         <v>64</v>
       </c>
-      <c r="E53" s="41">
-        <v>1</v>
-      </c>
-      <c r="F53" s="39"/>
-      <c r="G53" s="39"/>
-      <c r="H53" s="39"/>
-      <c r="I53" s="39">
+      <c r="E53" s="29">
+        <v>1</v>
+      </c>
+      <c r="F53" s="27"/>
+      <c r="G53" s="27"/>
+      <c r="H53" s="27"/>
+      <c r="I53" s="27">
         <f>E53*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>1</v>
       </c>
-      <c r="J53" s="40"/>
+      <c r="J53" s="28"/>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A54" s="39">
+      <c r="A54" s="27">
         <v>79562</v>
       </c>
-      <c r="B54" s="39" t="s">
-        <v>25</v>
-      </c>
-      <c r="C54" s="39">
+      <c r="B54" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="C54" s="27">
         <v>5818</v>
       </c>
-      <c r="D54" s="40" t="s">
+      <c r="D54" s="28" t="s">
         <v>28</v>
       </c>
-      <c r="E54" s="41">
-        <v>1</v>
-      </c>
-      <c r="F54" s="39"/>
-      <c r="G54" s="39"/>
-      <c r="H54" s="39"/>
-      <c r="I54" s="39">
+      <c r="E54" s="29">
+        <v>1</v>
+      </c>
+      <c r="F54" s="27"/>
+      <c r="G54" s="27"/>
+      <c r="H54" s="27"/>
+      <c r="I54" s="27">
         <f>E54*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>1</v>
       </c>
-      <c r="J54" s="40"/>
+      <c r="J54" s="28"/>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A55" s="39">
+      <c r="A55" s="27">
         <v>79563</v>
       </c>
-      <c r="B55" s="39" t="s">
-        <v>25</v>
-      </c>
-      <c r="C55" s="39">
+      <c r="B55" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="C55" s="27">
         <v>13302</v>
       </c>
-      <c r="D55" s="40" t="s">
+      <c r="D55" s="28" t="s">
         <v>29</v>
       </c>
-      <c r="E55" s="41">
-        <v>1</v>
-      </c>
-      <c r="F55" s="39"/>
-      <c r="G55" s="39"/>
-      <c r="H55" s="39"/>
-      <c r="I55" s="39">
+      <c r="E55" s="29">
+        <v>1</v>
+      </c>
+      <c r="F55" s="27"/>
+      <c r="G55" s="27"/>
+      <c r="H55" s="27"/>
+      <c r="I55" s="27">
         <f>E55*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>1</v>
       </c>
-      <c r="J55" s="40"/>
+      <c r="J55" s="28"/>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A56" s="39">
+      <c r="A56" s="27">
         <v>79582</v>
       </c>
-      <c r="B56" s="39" t="s">
-        <v>25</v>
-      </c>
-      <c r="C56" s="39">
+      <c r="B56" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="C56" s="27">
         <v>26088</v>
       </c>
-      <c r="D56" s="40" t="s">
+      <c r="D56" s="28" t="s">
         <v>46</v>
       </c>
-      <c r="E56" s="41">
-        <v>1</v>
-      </c>
-      <c r="F56" s="39"/>
-      <c r="G56" s="39"/>
-      <c r="H56" s="39"/>
-      <c r="I56" s="39">
+      <c r="E56" s="29">
+        <v>1</v>
+      </c>
+      <c r="F56" s="27"/>
+      <c r="G56" s="27"/>
+      <c r="H56" s="27"/>
+      <c r="I56" s="27">
         <f>E56*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>1</v>
       </c>
-      <c r="J56" s="40"/>
+      <c r="J56" s="28"/>
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A57" s="39">
+      <c r="A57" s="27">
         <v>79583</v>
       </c>
-      <c r="B57" s="39" t="s">
-        <v>25</v>
-      </c>
-      <c r="C57" s="39">
+      <c r="B57" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="C57" s="27">
         <v>26093</v>
       </c>
-      <c r="D57" s="40" t="s">
+      <c r="D57" s="28" t="s">
         <v>48</v>
       </c>
-      <c r="E57" s="41">
-        <v>1</v>
-      </c>
-      <c r="F57" s="39"/>
-      <c r="G57" s="39"/>
-      <c r="H57" s="39"/>
-      <c r="I57" s="39">
+      <c r="E57" s="29">
+        <v>1</v>
+      </c>
+      <c r="F57" s="27"/>
+      <c r="G57" s="27"/>
+      <c r="H57" s="27"/>
+      <c r="I57" s="27">
         <f>E57*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>1</v>
       </c>
-      <c r="J57" s="40"/>
+      <c r="J57" s="28"/>
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A58" s="39">
+      <c r="A58" s="27">
         <v>80709</v>
       </c>
-      <c r="B58" s="39" t="s">
-        <v>25</v>
-      </c>
-      <c r="C58" s="39">
+      <c r="B58" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="C58" s="27">
         <v>420279</v>
       </c>
-      <c r="D58" s="40" t="s">
+      <c r="D58" s="28" t="s">
         <v>65</v>
       </c>
-      <c r="E58" s="41">
-        <v>1</v>
-      </c>
-      <c r="F58" s="39"/>
-      <c r="G58" s="39"/>
-      <c r="H58" s="39"/>
-      <c r="I58" s="39">
+      <c r="E58" s="29">
+        <v>1</v>
+      </c>
+      <c r="F58" s="27"/>
+      <c r="G58" s="27"/>
+      <c r="H58" s="27"/>
+      <c r="I58" s="27">
         <f>E58*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>1</v>
       </c>
-      <c r="J58" s="40"/>
+      <c r="J58" s="28"/>
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A59" s="39">
+      <c r="A59" s="27">
         <v>79603</v>
       </c>
-      <c r="B59" s="39" t="s">
-        <v>25</v>
-      </c>
-      <c r="C59" s="39">
+      <c r="B59" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="C59" s="27">
         <v>421016</v>
       </c>
-      <c r="D59" s="40" t="s">
+      <c r="D59" s="28" t="s">
         <v>61</v>
       </c>
-      <c r="E59" s="41">
-        <v>1</v>
-      </c>
-      <c r="F59" s="39"/>
-      <c r="G59" s="39"/>
-      <c r="H59" s="39"/>
-      <c r="I59" s="39">
+      <c r="E59" s="29">
+        <v>1</v>
+      </c>
+      <c r="F59" s="27"/>
+      <c r="G59" s="27"/>
+      <c r="H59" s="27"/>
+      <c r="I59" s="27">
         <f>E59*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>1</v>
       </c>
-      <c r="J59" s="40"/>
+      <c r="J59" s="28"/>
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A60" s="39">
+      <c r="A60" s="27">
         <v>79604</v>
       </c>
-      <c r="B60" s="39" t="s">
-        <v>25</v>
-      </c>
-      <c r="C60" s="39">
+      <c r="B60" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="C60" s="27">
         <v>421072</v>
       </c>
-      <c r="D60" s="40" t="s">
+      <c r="D60" s="28" t="s">
         <v>66</v>
       </c>
-      <c r="E60" s="41">
-        <v>1</v>
-      </c>
-      <c r="F60" s="39"/>
-      <c r="G60" s="39"/>
-      <c r="H60" s="39"/>
-      <c r="I60" s="39">
+      <c r="E60" s="29">
+        <v>1</v>
+      </c>
+      <c r="F60" s="27"/>
+      <c r="G60" s="27"/>
+      <c r="H60" s="27"/>
+      <c r="I60" s="27">
         <f>E60*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>1</v>
       </c>
-      <c r="J60" s="40"/>
+      <c r="J60" s="28"/>
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A61" s="39">
+      <c r="A61" s="27">
         <v>79584</v>
       </c>
-      <c r="B61" s="39" t="s">
-        <v>25</v>
-      </c>
-      <c r="C61" s="39">
+      <c r="B61" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="C61" s="27">
         <v>26249</v>
       </c>
-      <c r="D61" s="40" t="s">
+      <c r="D61" s="28" t="s">
         <v>49</v>
       </c>
-      <c r="E61" s="41">
+      <c r="E61" s="29">
         <v>2</v>
       </c>
-      <c r="F61" s="39"/>
-      <c r="G61" s="39"/>
-      <c r="H61" s="39"/>
-      <c r="I61" s="39">
+      <c r="F61" s="27"/>
+      <c r="G61" s="27"/>
+      <c r="H61" s="27"/>
+      <c r="I61" s="27">
         <f>E61*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>2</v>
       </c>
-      <c r="J61" s="40"/>
+      <c r="J61" s="28"/>
     </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="10">
+    <mergeCell ref="D2:G2"/>
     <mergeCell ref="E9:F9"/>
     <mergeCell ref="G9:H9"/>
     <mergeCell ref="G5:H5"/>
@@ -2594,8 +2498,9 @@
     <mergeCell ref="I6:J6"/>
     <mergeCell ref="G7:H7"/>
     <mergeCell ref="I7:J7"/>
+    <mergeCell ref="D6:E6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>